<commit_message>
Alteração de componentes e anotações
</commit_message>
<xml_diff>
--- a/Componentes.xlsx
+++ b/Componentes.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://beontagbr-my.sharepoint.com/personal/joao_martins_beontag_com/Documents/Área de Trabalho/Projeto Aviso Baixa Tensão Utilizando LoRa/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="238" documentId="11_AD4D361C20488DEA4E38A04254587B545ADEDD90" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{326FBB01-64F9-4BFE-9797-AC641C61FAD8}"/>
+  <xr:revisionPtr revIDLastSave="313" documentId="11_AD4D361C20488DEA4E38A04254587B545ADEDD90" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3FDBF96A-AD2B-4538-9F77-D53049615E24}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="57">
   <si>
     <t>E32-433T20D</t>
   </si>
@@ -86,45 +86,9 @@
     <t>Buzzer</t>
   </si>
   <si>
-    <t>Sensor de tensão</t>
-  </si>
-  <si>
     <t>Placa fenolite (verificar o tamanho das placas)</t>
   </si>
   <si>
-    <t>https://www.jheletronico.com.br/pack-de-baterias-18650-li-ion-37v-104a-4-celulas-c-rabicho-2-fios</t>
-  </si>
-  <si>
-    <t>Bateria do leitor de tensão</t>
-  </si>
-  <si>
-    <t>Bateria 3.7V 10A</t>
-  </si>
-  <si>
-    <t>https://www.jheletronico.com.br/bateria-li-po-37v-21a-77wh-gsp7538868x</t>
-  </si>
-  <si>
-    <t>Bateria 3.7v 2100mah Litio</t>
-  </si>
-  <si>
-    <t>Bateria do receptor</t>
-  </si>
-  <si>
-    <t>Kit 10 Módulo Tp4056 Carregador De Bateria Usb Tipo C 5v 1a</t>
-  </si>
-  <si>
-    <t>Carregador de bateria</t>
-  </si>
-  <si>
-    <t>https://www.mercadolivre.com.br/kit-10-modulo-tp4056-carregador-de-bateria-usb-tipo-c-5v-1a/up/MLBU1741803625?pdp_filters=item_id:MLB3855613725#is_advertising=true&amp;searchVariation=MLBU1741803625&amp;backend_model=search-backend&amp;be_origin=backend&amp;position=8&amp;search_layout=grid&amp;type=pad&amp;tracking_id=90195325-382c-4867-9fed-c40bdb5dd9ef&amp;ad_domain=VQCATCORE_LST&amp;ad_position=8&amp;ad_click_id=ZjEzODkzMzQtZWZmOS00NWFkLWFiYjYtY2M2NTYyZjA4Y2Qz</t>
-  </si>
-  <si>
-    <t>Módulo Sensor De Tensão 0 a 250V AC - ZMPT101B</t>
-  </si>
-  <si>
-    <t>https://www.proesi.com.br/modulo-sensor-de-tens-o-ac-0-a-250vac-zmpt101b</t>
-  </si>
-  <si>
     <t>https://www.proesi.com.br/buzzer-5v-bip-continuo-pci-12mm-oscilador-interno</t>
   </si>
   <si>
@@ -206,9 +170,6 @@
     <t>Total/Item</t>
   </si>
   <si>
-    <t>Conector KK (definir)</t>
-  </si>
-  <si>
     <t>Terminal KK</t>
   </si>
   <si>
@@ -219,13 +180,41 @@
   </si>
   <si>
     <t>VALOR TOTAL</t>
+  </si>
+  <si>
+    <t>Sensor de Temperatura DS18B20</t>
+  </si>
+  <si>
+    <t>Sensor de Temperatura</t>
+  </si>
+  <si>
+    <t>https://www.proesi.com.br/conector-kk-3961-2-macho-3-96-mm-2-vias-180-graus</t>
+  </si>
+  <si>
+    <t>Conector 2 vias KK 3961 (para fonte)</t>
+  </si>
+  <si>
+    <t>Alojamento KK</t>
+  </si>
+  <si>
+    <t>Conector KK 5045 (definir)</t>
+  </si>
+  <si>
+    <t>Terminal KK (para fonte)</t>
+  </si>
+  <si>
+    <t>Alojamento 2 vias KK (para fonte)</t>
+  </si>
+  <si>
+    <t>https://www.proesi.com.br/sensor-de-temperatura-a-prova-d-agua-ds18b20</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
+    <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-[$R$-416]\ * #,##0.00_-;\-[$R$-416]\ * #,##0.00_-;_-[$R$-416]\ * &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
@@ -299,18 +288,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="3">
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
     <dxf>
       <font>
         <strike val="0"/>
@@ -324,9 +319,6 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-[$R$-416]\ * #,##0.00_-;\-[$R$-416]\ * #,##0.00_-;_-[$R$-416]\ * &quot;-&quot;??_-;_-@_-"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -342,8 +334,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{7A7C364E-ED0F-49A6-8597-0FDCA2B01F90}" name="Tabela2" displayName="Tabela2" ref="A1:H23" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:H23" xr:uid="{7A7C364E-ED0F-49A6-8597-0FDCA2B01F90}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{7A7C364E-ED0F-49A6-8597-0FDCA2B01F90}" name="Tabela2" displayName="Tabela2" ref="A1:H24" totalsRowShown="0" headerRowDxfId="2">
+  <autoFilter ref="A1:H24" xr:uid="{7A7C364E-ED0F-49A6-8597-0FDCA2B01F90}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{5F8A6799-28E9-45C8-A489-9682CB9D6F11}" name="Itens"/>
     <tableColumn id="2" xr3:uid="{5B6C232D-D070-4A53-A725-9164AB09EAB2}" name="Descrição"/>
@@ -351,8 +343,8 @@
     <tableColumn id="4" xr3:uid="{DDEBC4DC-8DF0-437E-BD1C-07E1E985BEAA}" name="Link Compra"/>
     <tableColumn id="5" xr3:uid="{FB7078F7-531E-4910-8A9A-FC0C08B18B2C}" name="Link Referência"/>
     <tableColumn id="6" xr3:uid="{737C8874-6B47-4565-9A0E-57E3F3112DA9}" name="Compra solicitada?"/>
-    <tableColumn id="7" xr3:uid="{E27E675F-CD59-4E96-AA6F-D6144E0C6A8D}" name="Valor unitário"/>
-    <tableColumn id="8" xr3:uid="{6CF4CF23-9FCC-482F-BA49-D624A2E2C8C3}" name="Total/Item" dataDxfId="1">
+    <tableColumn id="7" xr3:uid="{E27E675F-CD59-4E96-AA6F-D6144E0C6A8D}" name="Valor unitário" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{6CF4CF23-9FCC-482F-BA49-D624A2E2C8C3}" name="Total/Item" dataDxfId="0">
       <calculatedColumnFormula>C2*G2</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -623,52 +615,52 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.85546875" customWidth="1"/>
-    <col min="2" max="2" width="34.140625" customWidth="1"/>
+    <col min="2" max="2" width="35.7109375" customWidth="1"/>
     <col min="3" max="3" width="13.5703125" customWidth="1"/>
     <col min="4" max="4" width="15.7109375" customWidth="1"/>
     <col min="5" max="5" width="18.7109375" customWidth="1"/>
     <col min="6" max="6" width="21.85546875" customWidth="1"/>
-    <col min="7" max="7" width="17.7109375" customWidth="1"/>
-    <col min="8" max="8" width="14.42578125" customWidth="1"/>
+    <col min="7" max="7" width="17.7109375" style="6" customWidth="1"/>
+    <col min="8" max="8" width="14.42578125" style="6" customWidth="1"/>
     <col min="11" max="11" width="14.42578125" customWidth="1"/>
     <col min="12" max="12" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="K1" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="L1" s="6">
+      <c r="F1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="L1" s="5">
         <f>SUM(H2:H226)</f>
-        <v>1147.4299999999998</v>
+        <v>1080.1200000000003</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
@@ -688,12 +680,12 @@
         <v>6</v>
       </c>
       <c r="F2" t="s">
-        <v>53</v>
-      </c>
-      <c r="G2" s="3">
+        <v>41</v>
+      </c>
+      <c r="G2" s="6">
         <v>112.95</v>
       </c>
-      <c r="H2" s="3">
+      <c r="H2" s="6">
         <f>C2*G2</f>
         <v>338.85</v>
       </c>
@@ -713,12 +705,12 @@
       </c>
       <c r="E3" s="1"/>
       <c r="F3" t="s">
-        <v>53</v>
-      </c>
-      <c r="G3" s="3">
+        <v>41</v>
+      </c>
+      <c r="G3" s="6">
         <v>36</v>
       </c>
-      <c r="H3" s="3">
+      <c r="H3" s="6">
         <f t="shared" ref="H3:H23" si="0">C3*G3</f>
         <v>108</v>
       </c>
@@ -727,8 +719,7 @@
       <c r="B4" t="s">
         <v>11</v>
       </c>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3">
+      <c r="H4" s="6">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -737,8 +728,7 @@
       <c r="B5" t="s">
         <v>12</v>
       </c>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3">
+      <c r="H5" s="6">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -748,344 +738,314 @@
         <v>13</v>
       </c>
       <c r="E6" s="2"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3">
+      <c r="H6" s="6">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="B7" t="s">
         <v>15</v>
       </c>
       <c r="C7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="F7" t="s">
-        <v>53</v>
-      </c>
-      <c r="G7" s="3">
+        <v>41</v>
+      </c>
+      <c r="G7" s="6">
         <v>3.65</v>
       </c>
-      <c r="H7" s="3">
-        <f t="shared" si="0"/>
-        <v>7.3</v>
+      <c r="H7" s="6">
+        <f t="shared" si="0"/>
+        <v>10.95</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>17</v>
-      </c>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3">
+        <v>16</v>
+      </c>
+      <c r="H8" s="6">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="B9" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="C9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="F9" t="s">
-        <v>53</v>
-      </c>
-      <c r="G9" s="3">
+        <v>41</v>
+      </c>
+      <c r="G9" s="6">
         <v>70.45</v>
       </c>
-      <c r="H9" s="3">
-        <f t="shared" si="0"/>
-        <v>140.9</v>
+      <c r="H9" s="6">
+        <f t="shared" si="0"/>
+        <v>211.35000000000002</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" t="s">
         <v>20</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10">
+        <v>3</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C10">
-        <v>1</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>18</v>
-      </c>
       <c r="F10" t="s">
-        <v>53</v>
-      </c>
-      <c r="G10" s="3">
-        <v>79.900000000000006</v>
-      </c>
-      <c r="H10" s="3">
-        <f t="shared" si="0"/>
-        <v>79.900000000000006</v>
+        <v>41</v>
+      </c>
+      <c r="G10" s="6">
+        <v>84.31</v>
+      </c>
+      <c r="H10" s="6">
+        <f t="shared" si="0"/>
+        <v>252.93</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="B11" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C11">
         <v>1</v>
       </c>
-      <c r="D11" s="1" t="s">
-        <v>21</v>
+      <c r="D11" t="s">
+        <v>25</v>
       </c>
       <c r="F11" t="s">
-        <v>53</v>
-      </c>
-      <c r="G11" s="3">
-        <v>29.9</v>
-      </c>
-      <c r="H11" s="3">
-        <f t="shared" si="0"/>
-        <v>29.9</v>
+        <v>41</v>
+      </c>
+      <c r="G11" s="6">
+        <v>54.33</v>
+      </c>
+      <c r="H11" s="6">
+        <f t="shared" si="0"/>
+        <v>54.33</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="B12" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C12">
         <v>1</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="F12" t="s">
-        <v>53</v>
-      </c>
-      <c r="G12" s="3">
-        <v>31.87</v>
-      </c>
-      <c r="H12" s="3">
-        <f t="shared" si="0"/>
-        <v>31.87</v>
+        <v>41</v>
+      </c>
+      <c r="G12" s="6">
+        <v>21.58</v>
+      </c>
+      <c r="H12" s="6">
+        <f t="shared" si="0"/>
+        <v>21.58</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B13" t="s">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C13">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="F13" t="s">
-        <v>53</v>
-      </c>
-      <c r="G13" s="3">
-        <v>33.92</v>
-      </c>
-      <c r="H13" s="3">
-        <f t="shared" si="0"/>
-        <v>33.92</v>
+        <v>41</v>
+      </c>
+      <c r="G13" s="6">
+        <v>0.33</v>
+      </c>
+      <c r="H13" s="6">
+        <f t="shared" si="0"/>
+        <v>6.6000000000000005</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" t="s">
+        <v>34</v>
+      </c>
+      <c r="C14">
+        <v>20</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="F14" t="s">
         <v>41</v>
       </c>
-      <c r="B14" t="s">
-        <v>32</v>
-      </c>
-      <c r="C14">
-        <v>3</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="F14" t="s">
-        <v>53</v>
-      </c>
-      <c r="G14" s="3">
-        <v>84.31</v>
-      </c>
-      <c r="H14" s="3">
-        <f t="shared" si="0"/>
-        <v>252.93</v>
+      <c r="G14" s="6">
+        <v>0.22</v>
+      </c>
+      <c r="H14" s="6">
+        <f t="shared" si="0"/>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="B15" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="C15">
         <v>1</v>
       </c>
-      <c r="D15" t="s">
-        <v>37</v>
+      <c r="D15" s="1" t="s">
+        <v>32</v>
       </c>
       <c r="F15" t="s">
+        <v>41</v>
+      </c>
+      <c r="G15" s="6">
+        <v>40.25</v>
+      </c>
+      <c r="H15" s="6">
+        <f t="shared" si="0"/>
+        <v>40.25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
         <v>53</v>
       </c>
-      <c r="G15" s="3">
-        <v>54.33</v>
-      </c>
-      <c r="H15" s="3">
-        <f t="shared" si="0"/>
-        <v>54.33</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>49</v>
-      </c>
-      <c r="B16" t="s">
-        <v>39</v>
-      </c>
-      <c r="C16">
-        <v>1</v>
-      </c>
-      <c r="D16" s="1" t="s">
+      <c r="H16" s="6">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>44</v>
+      </c>
+      <c r="H17" s="6">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>52</v>
+      </c>
+      <c r="H18" s="6">
+        <f>C18*G18</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
+        <v>51</v>
+      </c>
+      <c r="C19">
+        <v>5</v>
+      </c>
+      <c r="D19" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="F16" t="s">
-        <v>53</v>
-      </c>
-      <c r="G16" s="3">
-        <v>21.58</v>
-      </c>
-      <c r="H16" s="3">
-        <f t="shared" si="0"/>
-        <v>21.58</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>52</v>
-      </c>
-      <c r="B17" t="s">
-        <v>42</v>
-      </c>
-      <c r="C17">
-        <v>10</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="F17" t="s">
-        <v>53</v>
-      </c>
-      <c r="G17" s="3">
-        <v>0.33</v>
-      </c>
-      <c r="H17" s="3">
-        <f t="shared" si="0"/>
-        <v>3.3000000000000003</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>48</v>
-      </c>
-      <c r="B18" t="s">
-        <v>46</v>
-      </c>
-      <c r="C18">
-        <v>20</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="F18" t="s">
-        <v>53</v>
-      </c>
-      <c r="G18" s="3">
-        <v>0.22</v>
-      </c>
-      <c r="H18" s="3">
-        <f t="shared" si="0"/>
-        <v>4.4000000000000004</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>45</v>
-      </c>
-      <c r="B19" t="s">
-        <v>43</v>
-      </c>
-      <c r="C19">
-        <v>1</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="F19" t="s">
-        <v>53</v>
-      </c>
-      <c r="G19" s="3">
-        <v>40.25</v>
-      </c>
-      <c r="H19" s="3">
-        <f t="shared" si="0"/>
-        <v>40.25</v>
+      <c r="H19" s="6">
+        <f>C19*G19</f>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
-        <v>56</v>
-      </c>
-      <c r="H20" s="3">
-        <f t="shared" si="0"/>
+        <v>54</v>
+      </c>
+      <c r="D20" s="1"/>
+      <c r="H20" s="6">
+        <f>C20*G20</f>
         <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
-        <v>57</v>
-      </c>
-      <c r="H21" s="3">
-        <f t="shared" si="0"/>
+        <v>55</v>
+      </c>
+      <c r="D21" s="1"/>
+      <c r="H21" s="6">
+        <f>C21*G21</f>
         <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
-        <v>58</v>
-      </c>
-      <c r="H22" s="3">
+        <v>45</v>
+      </c>
+      <c r="H22" s="6">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
-        <v>59</v>
-      </c>
-      <c r="H23" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <v>46</v>
+      </c>
+      <c r="H23" s="6">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>48</v>
+      </c>
+      <c r="B24" t="s">
+        <v>49</v>
+      </c>
+      <c r="C24">
+        <v>2</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F24" t="s">
+        <v>41</v>
+      </c>
+      <c r="G24" s="6">
+        <v>15.44</v>
+      </c>
+      <c r="H24" s="6">
+        <f>C24*G24</f>
+        <v>30.88</v>
       </c>
     </row>
   </sheetData>
@@ -1093,21 +1053,18 @@
     <hyperlink ref="E2" r:id="rId1" xr:uid="{AF6576B4-6DE2-47F3-8559-D5A91D757979}"/>
     <hyperlink ref="D3" r:id="rId2" xr:uid="{01B36D4B-6D0E-47CB-96AC-4049B6D85A8D}"/>
     <hyperlink ref="D2" r:id="rId3" xr:uid="{0EB90C2C-A82A-4CD9-80A7-8B30B1813239}"/>
-    <hyperlink ref="D10" r:id="rId4" xr:uid="{3A626835-A18E-4178-9C19-4C0D1E44D0B7}"/>
-    <hyperlink ref="D11" r:id="rId5" xr:uid="{48B4A9D6-D040-4A6A-AB7E-C8C45DD39535}"/>
-    <hyperlink ref="D12" r:id="rId6" location="is_advertising=true&amp;searchVariation=MLBU1741803625&amp;backend_model=search-backend&amp;be_origin=backend&amp;position=8&amp;search_layout=grid&amp;type=pad&amp;tracking_id=90195325-382c-4867-9fed-c40bdb5dd9ef&amp;ad_domain=VQCATCORE_LST&amp;ad_position=8&amp;ad_click_id=ZjEzODkzMzQtZWZmOS00NWFkLWFiYjYtY2M2NTYyZjA4Y2Qz" display="https://www.mercadolivre.com.br/kit-10-modulo-tp4056-carregador-de-bateria-usb-tipo-c-5v-1a/up/MLBU1741803625?pdp_filters=item_id:MLB3855613725#is_advertising=true&amp;searchVariation=MLBU1741803625&amp;backend_model=search-backend&amp;be_origin=backend&amp;position=8&amp;search_layout=grid&amp;type=pad&amp;tracking_id=90195325-382c-4867-9fed-c40bdb5dd9ef&amp;ad_domain=VQCATCORE_LST&amp;ad_position=8&amp;ad_click_id=ZjEzODkzMzQtZWZmOS00NWFkLWFiYjYtY2M2NTYyZjA4Y2Qz" xr:uid="{4648C704-A85C-4E18-9A4D-B1B2E0F39183}"/>
-    <hyperlink ref="D13" r:id="rId7" xr:uid="{7358FD83-19F7-4876-BB2E-AF7D8E9A48B3}"/>
-    <hyperlink ref="D7" r:id="rId8" xr:uid="{3D0F1949-FC6A-49BF-A365-12FB8436985F}"/>
-    <hyperlink ref="D14" r:id="rId9" xr:uid="{338E6731-18DD-4C88-8111-2780F5BE07E2}"/>
-    <hyperlink ref="D9" r:id="rId10" xr:uid="{53A34724-8848-4ED9-9BD7-A247EE9EEE2E}"/>
-    <hyperlink ref="D19" r:id="rId11" xr:uid="{A91FC859-90BA-4160-9975-AB6459E4F48C}"/>
-    <hyperlink ref="D18" r:id="rId12" xr:uid="{A79A0DF8-7266-4EE7-B0F4-2A155772603D}"/>
-    <hyperlink ref="D16" r:id="rId13" xr:uid="{E6A0DCFA-2996-419D-BD2B-163FA04EDDBE}"/>
-    <hyperlink ref="D17" r:id="rId14" xr:uid="{69097EAA-BFFC-4DD9-B95C-9D4B6E90193E}"/>
+    <hyperlink ref="D7" r:id="rId4" xr:uid="{3D0F1949-FC6A-49BF-A365-12FB8436985F}"/>
+    <hyperlink ref="D10" r:id="rId5" xr:uid="{338E6731-18DD-4C88-8111-2780F5BE07E2}"/>
+    <hyperlink ref="D9" r:id="rId6" xr:uid="{53A34724-8848-4ED9-9BD7-A247EE9EEE2E}"/>
+    <hyperlink ref="D15" r:id="rId7" xr:uid="{A91FC859-90BA-4160-9975-AB6459E4F48C}"/>
+    <hyperlink ref="D14" r:id="rId8" xr:uid="{A79A0DF8-7266-4EE7-B0F4-2A155772603D}"/>
+    <hyperlink ref="D12" r:id="rId9" xr:uid="{E6A0DCFA-2996-419D-BD2B-163FA04EDDBE}"/>
+    <hyperlink ref="D13" r:id="rId10" xr:uid="{69097EAA-BFFC-4DD9-B95C-9D4B6E90193E}"/>
+    <hyperlink ref="D19" r:id="rId11" xr:uid="{665AF76F-83AB-4E6A-8119-87760899E925}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId15"/>
+    <tablePart r:id="rId12"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>